<commit_message>
Update Length distribution of an object in its life history.xlsx
</commit_message>
<xml_diff>
--- a/Analysis/Length distribution of an object in its life history.xlsx
+++ b/Analysis/Length distribution of an object in its life history.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\GitHub\article\Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE84C475-99B4-45E2-A8B6-F443F4EDF459}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76A2188B-6C76-40B1-A26F-06F2C35BCF63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2842,7 +2842,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="00B050"/>
+              <a:srgbClr val="FFFF00"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -3860,7 +3860,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="FFFF00"/>
+              <a:srgbClr val="0070C0"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>

</xml_diff>